<commit_message>
#1 Completed and Fresh Deliverables Generated
</commit_message>
<xml_diff>
--- a/Design-Files/Button-Board_v1.0/Deliverables/BOM/Button-Board_v1.0.xlsx
+++ b/Design-Files/Button-Board_v1.0/Deliverables/BOM/Button-Board_v1.0.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20412"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Mars\Projects\Button-Board_v1.0\Design Files\Project Outputs for Button-Board_v1.0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eSpark Cons Group\Documents\GitHub\Melih-SoundSensor\bradfairman-ledproject\Design-Files\Button-Board_v1.0\Design File\Project Outputs for Button-Board\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B31EB40F-0C35-44D3-959D-75D5C8ADDD4D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="182">
   <si>
     <t>#</t>
   </si>
@@ -30,12 +31,12 @@
     <t>Capacitor</t>
   </si>
   <si>
-    <t>Diode</t>
-  </si>
-  <si>
     <t>FPC-1mm</t>
   </si>
   <si>
+    <t>Male Header</t>
+  </si>
+  <si>
     <t>Inductor</t>
   </si>
   <si>
@@ -45,28 +46,52 @@
     <t>Mosfet</t>
   </si>
   <si>
+    <t>Transistor</t>
+  </si>
+  <si>
     <t>Resistor</t>
   </si>
   <si>
-    <t>BATTERY CHARGER</t>
+    <t>Resistors</t>
+  </si>
+  <si>
+    <t>Switch</t>
   </si>
   <si>
     <t>IC</t>
   </si>
   <si>
+    <t>LED Driver</t>
+  </si>
+  <si>
+    <t>Optocouplers</t>
+  </si>
+  <si>
     <t>Designator</t>
   </si>
   <si>
-    <t>C1, C3, C4, C5, C8</t>
-  </si>
-  <si>
-    <t>C2, C6</t>
+    <t>C1, C8, C12</t>
+  </si>
+  <si>
+    <t>C2, C15</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>C4, C6, C9</t>
   </si>
   <si>
     <t>C7</t>
   </si>
   <si>
-    <t>D1</t>
+    <t>C10</t>
+  </si>
+  <si>
+    <t>C11</t>
+  </si>
+  <si>
+    <t>C13, C14</t>
   </si>
   <si>
     <t>J1, J3</t>
@@ -81,39 +106,51 @@
     <t>L1</t>
   </si>
   <si>
-    <t>LED3, LED4, LED5</t>
+    <t>L2</t>
+  </si>
+  <si>
+    <t>LED1, LED2, LED3</t>
   </si>
   <si>
     <t>Q1</t>
   </si>
   <si>
-    <t>R2, R5</t>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>R1, R3, R9, R12, R13, R17, R19, R20</t>
+  </si>
+  <si>
+    <t>R2, R7</t>
   </si>
   <si>
     <t>R4</t>
   </si>
   <si>
+    <t>R5</t>
+  </si>
+  <si>
     <t>R6</t>
   </si>
   <si>
-    <t>R7, R9, R12</t>
-  </si>
-  <si>
     <t>R8, R14, R15</t>
   </si>
   <si>
     <t>R10</t>
   </si>
   <si>
-    <t>R11</t>
-  </si>
-  <si>
-    <t>R13</t>
+    <t>R11, R21</t>
   </si>
   <si>
     <t>R16</t>
   </si>
   <si>
+    <t>R18</t>
+  </si>
+  <si>
+    <t>R22, R23</t>
+  </si>
+  <si>
     <t>SW1</t>
   </si>
   <si>
@@ -129,19 +166,40 @@
     <t>U4</t>
   </si>
   <si>
+    <t>U5</t>
+  </si>
+  <si>
+    <t>U6</t>
+  </si>
+  <si>
+    <t>U7</t>
+  </si>
+  <si>
     <t>Description</t>
   </si>
   <si>
-    <t>1 µF ±20% 6.3V Ceramic Capacitor X5R 0201 (0603 Metric), 1 µF ±10% 25V Ceramic Capacitor X5R 0402 (1005 Metric)</t>
-  </si>
-  <si>
-    <t>0.1 µF ±10% 16V Ceramic Capacitor X7R 0402 (1005 Metric)</t>
+    <t>1 µF ±20% 6.3V Ceramic Capacitor X5R 0201 (0603 Metric), CAP CER 1UF 25V X5R 0402</t>
+  </si>
+  <si>
+    <t>0.1 µF ±10% 16V Ceramic Capacitor X7R 0402 (1005 Metric), CAP CER 0.1UF 16V X7R 0402</t>
+  </si>
+  <si>
+    <t>CAP CER 4.7UF 16V X5R 0402</t>
+  </si>
+  <si>
+    <t>CAP CER 10UF 10V X5R 0402</t>
   </si>
   <si>
     <t>0.22 µF ±10% 25V Ceramic Capacitor X5R 0402 (1005 Metric)</t>
   </si>
   <si>
-    <t>DIODE ZENER 3.3V 200MW SOD323F</t>
+    <t>CAP CER 1UF 16V X5R 0201</t>
+  </si>
+  <si>
+    <t>CAP CER 2.2UF 10V X5R 0201</t>
+  </si>
+  <si>
+    <t>CAP CER 0.68UF 10V X5R 0402</t>
   </si>
   <si>
     <t>4 Position FFC, FPC Connector Contacts, Top and Bottom 0.039" (1.00mm) Surface Mount, Right Angle</t>
@@ -156,22 +214,31 @@
     <t>Inductor Power Shielded Wirewound 22uH 20% 100KHz Ferrite 1A 0.306Ohm DCR 1818 T/R</t>
   </si>
   <si>
-    <t>Green 520nm LED Indication - Discrete 3.2V 0603 (1608 Metric)</t>
+    <t>2.34A 1.5uH Shielded Power Inductors ±20% SMD Power Inductors ROHS</t>
+  </si>
+  <si>
+    <t>LED GREEN CLEAR CHIP SMD</t>
   </si>
   <si>
     <t>SOT-23 MOSFETs ROHS</t>
   </si>
   <si>
-    <t>27 kOhms ±1% 0.063W, 1/16W Chip Resistor 0402 (1005 Metric) Moisture Resistant Thick Film</t>
+    <t>TRANS NPN 40V 0.2A SOT523</t>
+  </si>
+  <si>
+    <t>10 kOhms ±1% 0.063W, 1/16W Chip Resistor 0402 (1005 Metric) Moisture Resistant Thick Film, RES 10K OHM 1% 1/16W 0402, RES SMD 10K OHM 0.1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>RES SMD 10K OHM 1% 1/20W 0201</t>
   </si>
   <si>
     <t>4.7 kOhms ±1% 0.063W, 1/16W Chip Resistor 0402 (1005 Metric) Moisture Resistant Thick Film</t>
   </si>
   <si>
-    <t>3 kOhms ±1% 0.063W, 1/16W Chip Resistor 0402 (1005 Metric) Moisture Resistant Thick Film</t>
-  </si>
-  <si>
-    <t>10 kOhms ±1% 0.063W, 1/16W Chip Resistor 0402 (1005 Metric) Moisture Resistant Thick Film</t>
+    <t>RES 0.01 OHM 1% 1W 1206</t>
+  </si>
+  <si>
+    <t>RES 470 OHM 1% 1/16W 0402</t>
   </si>
   <si>
     <t>100 Ohms ±1% 0.063W, 1/16W Chip Resistor 0402 (1005 Metric) Moisture Resistant Thick Film</t>
@@ -180,22 +247,25 @@
     <t>400 mOhms ±1% 0.25W, 1/4W Chip Resistor 1206 (3216 Metric) Automotive AEC-Q200, Current Sense, Moisture Resistant Thick Film</t>
   </si>
   <si>
-    <t>1 kOhms ±1% 0.063W, 1/16W Chip Resistor 0402 (1005 Metric) Moisture Resistant Thick Film</t>
-  </si>
-  <si>
-    <t>7.68 kOhms ±1% 0.063W, 1/16W Chip Resistor 0402 (1005 Metric) Automotive AEC-Q200, Moisture Resistant Thick Film</t>
-  </si>
-  <si>
-    <t>20 Ohms ±1% 0.2W, 1/5W Chip Resistor 0402 (1005 Metric) Automotive AEC-Q200, Pulse Withstanding Thick Film</t>
-  </si>
-  <si>
-    <t>Tactile Switch SPST-NO Top Actuated Surface Mount</t>
-  </si>
-  <si>
-    <t>Charger IC Multi-Chemistry 8-WSON (2x2)</t>
-  </si>
-  <si>
-    <t>IC REG LDO 3.3V 0.25A SOT23-3</t>
+    <t>1 kOhms ±1% 0.063W, 1/16W Chip Resistor 0402 (1005 Metric) Moisture Resistant Thick Film, RES 1K OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>RES 10 OHM 1% 1/4W 1206</t>
+  </si>
+  <si>
+    <t>RES SMD 10K OHM 0.1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>RES 4.7K OHM 1% 1/20W 0201</t>
+  </si>
+  <si>
+    <t>No Gull Wing 50mA 100MΩ 80000 260gf@±50gf 12V -25℃~+85℃ 1.7mm Golden Round Button Brick nogging SPST SMD Tactile Switches ROHS</t>
+  </si>
+  <si>
+    <t>4.5V~5.5V 锂离子/Polymer 1 600mA SOT-23-5 Battery Management ICs ROHS</t>
+  </si>
+  <si>
+    <t>IC PB ON/OFF CONTROLLER TSOT23-8</t>
   </si>
   <si>
     <t>AVR tinyAVR™ 1, Functional Safety (FuSa) Microcontroller IC 8-Bit 20MHz 16KB (16K x 8) FLASH 20-VQFN (3x3)</t>
@@ -204,13 +274,19 @@
     <t>LED Driver IC 1 Output DC DC Regulator Step-Up (Boost) PWM Dimming 550mA (Switch) SOT-23-6</t>
   </si>
   <si>
+    <t>IC FUEL GAUGE LI-ION 1CL 9DSBGA</t>
+  </si>
+  <si>
+    <t>OPTOISOLATOR 3.75KV TRANS 4-SOP</t>
+  </si>
+  <si>
     <t>Footprint</t>
   </si>
   <si>
     <t>Cap-0402</t>
   </si>
   <si>
-    <t>SOD323F</t>
+    <t>CAP-0201</t>
   </si>
   <si>
     <t>XF3M(1)-0415-1B</t>
@@ -225,25 +301,34 @@
     <t>IND_1235AS-H-220M=P3</t>
   </si>
   <si>
-    <t>150060GS75000</t>
+    <t>LVT303012-1R5M-N</t>
+  </si>
+  <si>
+    <t>LED-0402</t>
   </si>
   <si>
     <t>SOT-23</t>
   </si>
   <si>
+    <t>SOT-523</t>
+  </si>
+  <si>
     <t>Res-0402</t>
   </si>
   <si>
+    <t>Res-0201</t>
+  </si>
+  <si>
     <t>Res-1206</t>
   </si>
   <si>
-    <t>RESC1005X40N</t>
-  </si>
-  <si>
-    <t>PTS525SM15SMTR2LFS</t>
-  </si>
-  <si>
-    <t>BQ25170DSGR</t>
+    <t>TC-0522C-1.7-260G_</t>
+  </si>
+  <si>
+    <t>SOT-23-5</t>
+  </si>
+  <si>
+    <t>TSOT-23-8</t>
   </si>
   <si>
     <t>20-VQFN (3x3)</t>
@@ -252,16 +337,40 @@
     <t>AP3019AKTR-G1</t>
   </si>
   <si>
+    <t>DSBGA-9 (1.651x1.61)</t>
+  </si>
+  <si>
+    <t>SON-10-EP(2.5x2.5)</t>
+  </si>
+  <si>
+    <t>SOP-4-1.27mm pitch Body 2.6mm</t>
+  </si>
+  <si>
     <t>Manufacturer Part Number</t>
   </si>
   <si>
-    <t>GRM155R71C104KA88J</t>
+    <t>GRM033R60J105MEA2D, GRM155R61E105KA12D</t>
+  </si>
+  <si>
+    <t>GRM155R71C104KA88J, GRM155R71C104KA88D</t>
+  </si>
+  <si>
+    <t>CL05A475MO5NUNC</t>
+  </si>
+  <si>
+    <t>CL05A106MP5NUNC</t>
   </si>
   <si>
     <t>CC0402KRX5R8BB224</t>
   </si>
   <si>
-    <t>MM3Z3V3B</t>
+    <t>CC0201MRX5R7BB105</t>
+  </si>
+  <si>
+    <t>CC0201MRX5R6BB225</t>
+  </si>
+  <si>
+    <t>CC0402KRX5R6BB684</t>
   </si>
   <si>
     <t>SM02B-SRSS-TB_LF__SN_</t>
@@ -273,19 +382,28 @@
     <t>1235AS-H-220M=P3</t>
   </si>
   <si>
+    <t>XZVG68W-2</t>
+  </si>
+  <si>
     <t>FDN335N</t>
   </si>
   <si>
-    <t>RC0402FR-0727KL</t>
+    <t>MMBT3904T-7-F</t>
+  </si>
+  <si>
+    <t>RC0402FR-0710KL, RT0402BRD0710KL</t>
+  </si>
+  <si>
+    <t>RC0201FR-0710KL</t>
   </si>
   <si>
     <t>RC0402FR-074K7L</t>
   </si>
   <si>
-    <t>RC0402FR-073KL</t>
-  </si>
-  <si>
-    <t>RC0402FR-0710KL</t>
+    <t>PA1206FRE470R01Z</t>
+  </si>
+  <si>
+    <t>RC0402FR-07470RL</t>
   </si>
   <si>
     <t>RC0402FR-07100RL</t>
@@ -297,61 +415,88 @@
     <t>RC0402FR-071KL</t>
   </si>
   <si>
-    <t>AC0402FR-077K68L</t>
-  </si>
-  <si>
-    <t>RCS040220R0FKED</t>
-  </si>
-  <si>
-    <t>PTS526 SK15 SMTR2 LFS</t>
-  </si>
-  <si>
-    <t>MCP1700T-3302E/TT</t>
+    <t>RC1206FR-0710RL</t>
+  </si>
+  <si>
+    <t>RT0402BRD0710KL</t>
+  </si>
+  <si>
+    <t>RC0201FR-074K7L</t>
+  </si>
+  <si>
+    <t>TC-0522C-1.7-260G</t>
+  </si>
+  <si>
+    <t>TP4054</t>
+  </si>
+  <si>
+    <t>LTC2950CTS8-1#TRPBF</t>
   </si>
   <si>
     <t>ATTINY1616-MNR</t>
   </si>
   <si>
+    <t>BQ27426YZFR</t>
+  </si>
+  <si>
+    <t>TCMT1107</t>
+  </si>
+  <si>
     <t>Manufacturer</t>
   </si>
   <si>
+    <t>Murata Electronics, Murata</t>
+  </si>
+  <si>
+    <t>Samsung</t>
+  </si>
+  <si>
+    <t>YAGEO</t>
+  </si>
+  <si>
+    <t>Yageo</t>
+  </si>
+  <si>
+    <t>Omron Electronics Inc-EMC Div</t>
+  </si>
+  <si>
+    <t>JST Sales</t>
+  </si>
+  <si>
     <t>Murata Electronics</t>
   </si>
   <si>
-    <t>YAGEO</t>
-  </si>
-  <si>
-    <t>ON Semiconductor / Fairchild</t>
-  </si>
-  <si>
-    <t>Omron Electronics Inc-EMC Div</t>
-  </si>
-  <si>
-    <t>JST Sales</t>
-  </si>
-  <si>
-    <t>Würth Elektronik</t>
+    <t>Chilisin Elec</t>
+  </si>
+  <si>
+    <t>SunLED</t>
   </si>
   <si>
     <t>onsemi</t>
   </si>
   <si>
-    <t>Vishay Dale</t>
-  </si>
-  <si>
-    <t>C&amp;K</t>
+    <t>Diodes Zetex</t>
+  </si>
+  <si>
+    <t>HCTL</t>
+  </si>
+  <si>
+    <t>TPOWER</t>
+  </si>
+  <si>
+    <t>Analog Devices / Linear Technology</t>
+  </si>
+  <si>
+    <t>Microchip Tech</t>
+  </si>
+  <si>
+    <t>Diodes Incorporated</t>
   </si>
   <si>
     <t>Texas Instruments</t>
   </si>
   <si>
-    <t>Microchip</t>
-  </si>
-  <si>
-    <t>Microchip Tech</t>
-  </si>
-  <si>
-    <t>Diodes Incorporated</t>
+    <t>Vishay Semiconductors</t>
   </si>
   <si>
     <t>Comment</t>
@@ -363,25 +508,37 @@
     <t>0.1uF</t>
   </si>
   <si>
+    <t>4.7uF</t>
+  </si>
+  <si>
+    <t>10uF</t>
+  </si>
+  <si>
     <t>0.22uF</t>
   </si>
   <si>
+    <t>2.2uF</t>
+  </si>
+  <si>
+    <t>680nF</t>
+  </si>
+  <si>
     <t>22uH</t>
   </si>
   <si>
-    <t>GREEN</t>
-  </si>
-  <si>
-    <t>27K</t>
+    <t>1.5uH</t>
+  </si>
+  <si>
+    <t>10K</t>
   </si>
   <si>
     <t>4.7K</t>
   </si>
   <si>
-    <t>3K</t>
-  </si>
-  <si>
-    <t>10K</t>
+    <t>10mR</t>
+  </si>
+  <si>
+    <t>470R</t>
   </si>
   <si>
     <t>100R</t>
@@ -393,34 +550,28 @@
     <t>1K</t>
   </si>
   <si>
-    <t>7.68K</t>
-  </si>
-  <si>
-    <t>20R</t>
+    <t>10R</t>
+  </si>
+  <si>
+    <t>NC</t>
+  </si>
+  <si>
+    <t>TPS63031DSKR</t>
   </si>
   <si>
     <t>Quantity</t>
   </si>
   <si>
-    <t>0402X105K250CT</t>
-  </si>
-  <si>
-    <t>Walsin Technologies</t>
-  </si>
-  <si>
-    <t>Header</t>
-  </si>
-  <si>
-    <t>Switch</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Remarks</t>
+    <t>connector</t>
+  </si>
+  <si>
+    <t>IC REG BUCK-BST 3v3 900MA 10SON</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -905,9 +1056,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -915,14 +1066,13 @@
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -933,9 +1083,8 @@
       <c r="H1" s="2"/>
       <c r="I1" s="14"/>
       <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -944,31 +1093,28 @@
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>61</v>
+        <v>86</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>77</v>
+        <v>108</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>97</v>
+        <v>140</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>111</v>
+        <v>159</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -978,433 +1124,420 @@
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>62</v>
+        <v>87</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>112</v>
+        <v>160</v>
       </c>
       <c r="J3" s="7">
-        <v>5</v>
-      </c>
-      <c r="K3" s="7"/>
-    </row>
-    <row r="4" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B26" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B36" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>62</v>
+        <v>87</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>78</v>
+        <v>110</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>98</v>
+        <v>141</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>113</v>
+        <v>161</v>
       </c>
       <c r="J4" s="9">
         <v>2</v>
       </c>
-      <c r="K4" s="9"/>
-    </row>
-    <row r="5" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="11">
         <f>ROW(B5) - ROW($B$2)</f>
         <v>3</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="13" t="s">
         <v>2</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>62</v>
+        <v>87</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>79</v>
+        <v>111</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>99</v>
+        <v>142</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>114</v>
+        <v>162</v>
       </c>
       <c r="J5" s="7">
         <v>1</v>
       </c>
-      <c r="K5" s="7"/>
-    </row>
-    <row r="6" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="11">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C6" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="J6" s="9">
         <v>3</v>
       </c>
-      <c r="D6" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="I6" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="J6" s="9">
-        <v>1</v>
-      </c>
-      <c r="K6" s="9"/>
-    </row>
-    <row r="7" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
         <v>5</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>64</v>
+        <v>113</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>101</v>
+        <v>143</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>64</v>
+        <v>164</v>
       </c>
       <c r="J7" s="7">
-        <v>2</v>
-      </c>
-      <c r="K7" s="7"/>
-    </row>
-    <row r="8" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="11">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>129</v>
+        <v>2</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>81</v>
+        <v>114</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>102</v>
+        <v>144</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>65</v>
+        <v>160</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
       </c>
-      <c r="K8" s="9"/>
-    </row>
-    <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="11">
         <f>ROW(B9) - ROW($B$2)</f>
         <v>7</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>129</v>
+        <v>2</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>66</v>
+        <v>88</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="H9" s="7"/>
+        <v>115</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>144</v>
+      </c>
       <c r="I9" s="8" t="s">
-        <v>66</v>
+        <v>165</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
       </c>
-      <c r="K9" s="7"/>
-    </row>
-    <row r="10" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>67</v>
+        <v>87</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>83</v>
+        <v>116</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>98</v>
+        <v>144</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>115</v>
+        <v>166</v>
       </c>
       <c r="J10" s="9">
-        <v>1</v>
-      </c>
-      <c r="K10" s="9"/>
-    </row>
-    <row r="11" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="11">
         <f>ROW(B11) - ROW($B$2)</f>
         <v>9</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>68</v>
+        <v>89</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>68</v>
+        <v>89</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>103</v>
+        <v>145</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>116</v>
+        <v>89</v>
       </c>
       <c r="J11" s="7">
-        <v>3</v>
-      </c>
-      <c r="K11" s="7"/>
-    </row>
-    <row r="12" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>7</v>
+        <v>180</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>84</v>
+        <v>117</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>104</v>
+        <v>146</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
       </c>
-      <c r="K12" s="9"/>
-    </row>
-    <row r="13" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
         <v>11</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>99</v>
-      </c>
+        <v>118</v>
+      </c>
+      <c r="H13" s="7"/>
       <c r="I13" s="8" t="s">
-        <v>117</v>
+        <v>91</v>
       </c>
       <c r="J13" s="7">
-        <v>2</v>
-      </c>
-      <c r="K13" s="7"/>
-    </row>
-    <row r="14" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="11">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>70</v>
+        <v>92</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>86</v>
+        <v>119</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>99</v>
+        <v>147</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>118</v>
+        <v>167</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
       </c>
-      <c r="K14" s="9"/>
-    </row>
-    <row r="15" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
         <f>ROW(B15) - ROW($B$2)</f>
         <v>13</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>99</v>
+        <v>148</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>119</v>
+        <v>168</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
       </c>
-      <c r="K15" s="7"/>
-    </row>
-    <row r="16" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>70</v>
+        <v>94</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>88</v>
+        <v>120</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>99</v>
+        <v>149</v>
       </c>
       <c r="I16" s="10" t="s">
         <v>120</v>
@@ -1412,41 +1545,39 @@
       <c r="J16" s="9">
         <v>3</v>
       </c>
-      <c r="K16" s="9"/>
-    </row>
-    <row r="17" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
         <v>15</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>89</v>
+        <v>121</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>99</v>
+        <v>150</v>
       </c>
       <c r="I17" s="8" t="s">
         <v>121</v>
       </c>
       <c r="J17" s="7">
-        <v>3</v>
-      </c>
-      <c r="K17" s="7"/>
-    </row>
-    <row r="18" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
@@ -1456,19 +1587,19 @@
         <v>8</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>90</v>
+        <v>122</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>99</v>
+        <v>151</v>
       </c>
       <c r="I18" s="10" t="s">
         <v>122</v>
@@ -1476,137 +1607,132 @@
       <c r="J18" s="9">
         <v>1</v>
       </c>
-      <c r="K18" s="9"/>
-    </row>
-    <row r="19" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:10" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
         <v>17</v>
       </c>
       <c r="C19" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="I19" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="J19" s="7">
         <v>8</v>
       </c>
-      <c r="D19" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="G19" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="I19" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="J19" s="7">
-        <v>1</v>
-      </c>
-      <c r="K19" s="7"/>
-    </row>
-    <row r="20" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="20" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>99</v>
+        <v>144</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>124</v>
+        <v>169</v>
       </c>
       <c r="J20" s="9">
-        <v>1</v>
-      </c>
-      <c r="K20" s="9"/>
-    </row>
-    <row r="21" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
         <f>ROW(B21) - ROW($B$2)</f>
         <v>19</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>72</v>
+        <v>97</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>93</v>
+        <v>125</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>105</v>
+        <v>143</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>125</v>
+        <v>170</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
       </c>
-      <c r="K21" s="7"/>
-    </row>
-    <row r="22" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>56</v>
+        <v>71</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>73</v>
+        <v>99</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>94</v>
+        <v>126</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>106</v>
+        <v>144</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>94</v>
+        <v>171</v>
       </c>
       <c r="J22" s="9">
         <v>1</v>
       </c>
-      <c r="K22" s="9"/>
-    </row>
-    <row r="23" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
         <f>ROW(B23) - ROW($B$2)</f>
@@ -1616,127 +1742,464 @@
         <v>9</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>74</v>
+        <v>127</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>74</v>
+        <v>172</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
       </c>
-      <c r="K23" s="7"/>
-    </row>
-    <row r="24" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="11">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>108</v>
+        <v>143</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>95</v>
+        <v>173</v>
       </c>
       <c r="J24" s="9">
-        <v>1</v>
-      </c>
-      <c r="K24" s="9"/>
-    </row>
-    <row r="25" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="11">
         <f>ROW(B25) - ROW($B$2)</f>
         <v>23</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>96</v>
+        <v>129</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>109</v>
+        <v>143</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>96</v>
+        <v>174</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
       </c>
-      <c r="K25" s="7"/>
-    </row>
-    <row r="26" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="11">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D26" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E26" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="G26" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="H26" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="I26" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="J26" s="9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="1"/>
+      <c r="B27" s="11">
+        <f>ROW(B27) - ROW($B$2)</f>
+        <v>25</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="I27" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="J27" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="1"/>
+      <c r="B28" s="11">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E28" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="G28" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="I28" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="J28" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="1"/>
+      <c r="B29" s="11">
+        <f>ROW(B29) - ROW($B$2)</f>
+        <v>27</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G29" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="I29" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="J29" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="1"/>
+      <c r="B30" s="11">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E30" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="G30" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="H30" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="I30" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="J30" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="1"/>
+      <c r="B31" s="11">
+        <f>ROW(B31) - ROW($B$2)</f>
+        <v>29</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="G31" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I31" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="J31" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="1"/>
+      <c r="B32" s="11">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="E32" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="G32" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="H32" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="I32" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="J32" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="1"/>
+      <c r="B33" s="11">
+        <f>ROW(B33) - ROW($B$2)</f>
+        <v>31</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="G33" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="I33" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="J33" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="1"/>
+      <c r="B34" s="11">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E34" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="G34" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="H34" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="I34" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="J34" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="1"/>
+      <c r="B35" s="11">
+        <f>ROW(B35) - ROW($B$2)</f>
+        <v>33</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="G35" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="H35" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="I35" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="J35" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="1"/>
+      <c r="B36" s="11">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E36" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="G36" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="H36" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="I36" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="J36" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="1"/>
+      <c r="B37" s="11">
+        <f>ROW(B37) - ROW($B$2)</f>
         <v>35</v>
       </c>
-      <c r="E26" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="F26" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="G26" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="H26" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="I26" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="J26" s="9">
-        <v>1</v>
-      </c>
-      <c r="K26" s="9"/>
+      <c r="C37" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="G37" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="I37" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="J37" s="7">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="I1:J1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>